<commit_message>
Group B: 6900 SPEC (male ORB x female NPSM swivel, existing ends) + A3 table correction: 22 configurations generate, checks clean
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6900.xlsx
+++ b/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6900.xlsx
@@ -465,7 +465,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OMi 6900 Female Adapter Union x Male NPSM - Design Table v1 | AW s105 double-pass 24 rows | female-JIC internals are the open lookup | GENERATED 2026-09-06</t>
+          <t>OMi 6900 Male ORB x Female NPSM Swivel Adapter - Design Table v1 | AW s105 double-pass 24 rows | GENERATED 2026-09-06 | identity corrected 2026-10-21 (A3 2026-10-18; was "Female Adapter Union x Male NPSM")</t>
         </is>
       </c>
     </row>
@@ -580,12 +580,12 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>7/16-20 (female JIC union) x 1/8-27 NPSM</t>
+          <t>7/16-20 (male ORB) x 1/8-27 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.09 vs Brennan L 1.14; L2 0.94 vs Brennan L1 1.0; D 0.13 vs Brennan A2D 0.15</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -643,12 +643,12 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>7/16-20 (female JIC union) x 1/4-18 NPSM</t>
+          <t>7/16-20 (male ORB) x 1/4-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): agree within the 2-decimal rounding on W4 / L2 / C2 / C / D1 / D</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -706,12 +706,12 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>7/16-20 (female JIC union) x 3/8-18 NPSM</t>
+          <t>7/16-20 (male ORB) x 3/8-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.39 vs Brennan L 1.36</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -742,10 +742,10 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1.3</v>
+        <v>1.28</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1.19</v>
+        <v>1.09</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.63</v>
@@ -769,22 +769,22 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>1/2-20 (female JIC union) x 1/4-18 NPSM</t>
+          <t>1/2-20 (male ORB) x 1/4-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Air-Way s105 only (double-pass 24 rows); NPSM male end fully published</t>
+          <t>[BRENNAN-CELL 2026-10-21: W4@DRIVE, L2@DRIVE] Air-Way s105 only (double-pass 24 rows); NPSM male end fully published</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.3 vs Brennan L 1.28; L2 1.19 vs Brennan L1 1.09 | Q-CONFLICT-6900-05-04-O: Air-Way W4 1.3 / L2 1.19 put the nut face 0.11 from the stem tip - the measured -04 NPSM swivel cannot be built (nut / stem order; Brennan 1404-04: 0.19) -&gt; both cells = the Brennan CAD record L 1.28 / L1 1.09 (user Q1 2026-10-20 "use brennans"; 2026-10-18 recommendation was "keep W4" - tell the user)</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -795,6 +795,11 @@
       <c r="O6" t="inlineStr">
         <is>
           <t>6900-05-04-O</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
         </is>
       </c>
     </row>
@@ -832,12 +837,12 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>9/16-18 (female JIC union) x 1/4-18 NPSM</t>
+          <t>9/16-18 (male ORB) x 1/4-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -847,7 +852,7 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.36 vs Brennan L 1.26; L2 1.17 vs Brennan L1 1.07</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -895,12 +900,12 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>9/16-18 (female JIC union) x 3/8-18 NPSM</t>
+          <t>9/16-18 (male ORB) x 3/8-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -910,7 +915,7 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.42 vs Brennan L 1.46</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -958,12 +963,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>9/16-18 (female JIC union) x 1/2-14 NPSM</t>
+          <t>9/16-18 (male ORB) x 1/2-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -973,7 +978,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: L2 1.23 vs Brennan L1 1.29; C2HEX 0.88 vs Brennan C4 0.812</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1021,12 +1026,12 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>3/4-16 (female JIC union) x 1/4-18 NPSM</t>
+          <t>3/4-16 (male ORB) x 1/4-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -1036,7 +1041,7 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.42 vs Brennan L 1.36; L2 1.23 vs Brennan L1 1.17</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1084,12 +1089,12 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>3/4-16 (female JIC union) x 3/8-18 NPSM</t>
+          <t>3/4-16 (male ORB) x 3/8-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1099,7 +1104,7 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.48 vs Brennan L 1.4</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1147,12 +1152,12 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>3/4-16 (female JIC union) x 1/2-14 NPSM</t>
+          <t>3/4-16 (male ORB) x 1/2-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
@@ -1162,7 +1167,7 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.61 vs Brennan L 1.55</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1210,12 +1215,12 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>3/4-16 (female JIC union) x 3/4-14 NPSM</t>
+          <t>3/4-16 (male ORB) x 3/4-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1225,7 +1230,7 @@
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.74 vs Brennan L 1.76</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1273,12 +1278,12 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>7/8-14 (female JIC union) x 3/8-18 NPSM</t>
+          <t>7/8-14 (male ORB) x 3/8-18 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1288,7 +1293,7 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.62 vs Brennan L 1.47; L2 1.37 vs Brennan L1 1.26</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1336,12 +1341,12 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>7/8-14 (female JIC union) x 1/2-14 NPSM</t>
+          <t>7/8-14 (male ORB) x 1/2-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -1351,7 +1356,7 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.73 vs Brennan L 1.61</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1399,12 +1404,12 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>7/8-14 (female JIC union) x 3/4-14 NPSM</t>
+          <t>7/8-14 (male ORB) x 3/4-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -1414,7 +1419,7 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.88 vs Brennan L 1.72; L2 1.55 vs Brennan L1 1.37; D 0.48 vs Brennan A2D 0.635</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1462,12 +1467,12 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>1 1/16-12 (female JIC union) x 1/2-14 NPSM</t>
+          <t>1 1/16-12 (male ORB) x 1/2-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -1477,7 +1482,7 @@
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.78 vs Brennan L 1.73</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1525,12 +1530,12 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>1 1/16-12 (female JIC union) x 3/4-14 NPSM</t>
+          <t>1 1/16-12 (male ORB) x 3/4-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
@@ -1540,7 +1545,7 @@
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 1.91 vs Brennan L 1.95; L2 1.58 vs Brennan L1 1.6</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1588,12 +1593,12 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>1 1/16-12 (female JIC union) x 1-11 1/2 NPSM</t>
+          <t>1 1/16-12 (male ORB) x 1-11 1/2 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -1603,7 +1608,7 @@
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: L2 1.66 vs Brennan L1 1.7; D 0.84 vs Brennan A2D 0.78</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1709,12 +1714,12 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>1 5/16-12 (female JIC union) x 3/4-14 NPSM</t>
+          <t>1 5/16-12 (male ORB) x 3/4-14 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -1724,7 +1729,7 @@
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 2.06 vs Brennan L 2.08</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1772,12 +1777,12 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>1 5/16-12 (female JIC union) x 1-11 1/2 NPSM</t>
+          <t>1 5/16-12 (male ORB) x 1-11 1/2 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
@@ -1787,7 +1792,7 @@
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 2.13 vs Brennan L 2.06; L2 1.75 vs Brennan L1 1.71</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1951,12 +1956,12 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>1 5/8-12 (female JIC union) x 1 1/4-11 1/2 NPSM</t>
+          <t>1 5/8-12 (male ORB) x 1 1/4-11 1/2 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -1966,7 +1971,7 @@
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): differ: W4 2.32 vs Brennan L 2.21; L2 1.89 vs Brennan L1 1.79; D1 1.08 vs Brennan B1D 1.01</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2014,12 +2019,12 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>1 7/8-12 (female JIC union) x 1 1/2-11 1/2 NPSM</t>
+          <t>1 7/8-12 (male ORB) x 1 1/2-11 1/2 NPSM (female swivel)</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
@@ -2029,7 +2034,7 @@
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: female-JIC union internal geometry UNPUBLISHED (nut thread depth, cone seat) - same lookup blocking 2406; measure a Brennan STEP</t>
+          <t>A3 (user 2026-10-18): male ORB x female NPSM swivel straight - the old "female-JIC union internals" block was the wrong identity (removed 2026-10-21) | Brennan CAD record cross-check (2026-10-21; Air-Way values built): agree within the 2-decimal rounding on W4 / L2 / C2 / C / D1 / D</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2049,6 +2054,12 @@
           <t>6900-32-32-O</t>
         </is>
       </c>
+      <c r="B27" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
       <c r="D27" t="n">
         <v>2.75</v>
       </c>
@@ -2058,6 +2069,9 @@
       <c r="F27" t="n">
         <v>1.781</v>
       </c>
+      <c r="G27" t="n">
+        <v>1.781</v>
+      </c>
       <c r="H27" t="n">
         <v>2.5</v>
       </c>
@@ -2066,6 +2080,11 @@
           <t>6900-32-32-O</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2 1/2-12 (male ORB) x 2-11 1/2 NPSM (female swivel)</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>ASSUMED</t>
@@ -2073,12 +2092,12 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: C2HEX@HEX, CHEX@HEX, D1@BORE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: W4@DRIVE, L2@DRIVE, D@BORE] [BRENNAN-CAD 2026-10-21: C2HEX@HEX, CHEX@HEX, D1@BORE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 6900-32-32-O (PARTcommunity / CADENAS, C2HEX@HEX=C4, CHEX@HEX=C, D1@BORE=B1D, THDMAJ_B@DRIVE=B1THD; user 2026-10-21 "yes you can use them following my rule")</t>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 6900-32-32-O (PARTcommunity / CADENAS, C2HEX@HEX=C4, CHEX@HEX=C, D1@BORE=B1D, THDMAJ_B@DRIVE=B1THD; user 2026-10-21 "yes you can use them following my rule") | Brennan CAD record 6900-32-32-O (PARTcommunity / CADENAS, group B 2026-10-21: W4@DRIVE=L, L2@DRIVE=L1, D@BORE=A2D; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">

</xml_diff>